<commit_message>
:boar: filtering clusters before rarefying (on all the physeq object)
</commit_message>
<xml_diff>
--- a/data/derived_data/2_RarefyData/ps_rare_ITS_sample_data.xlsx
+++ b/data/derived_data/2_RarefyData/ps_rare_ITS_sample_data.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="373" uniqueCount="373">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="372" uniqueCount="372">
   <si>
     <t xml:space="preserve"/>
   </si>
@@ -789,9 +789,6 @@
   </si>
   <si>
     <t xml:space="preserve">MS_166</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MS_167</t>
   </si>
   <si>
     <t xml:space="preserve">MS_168</t>
@@ -10601,7 +10598,7 @@
         <v>238</v>
       </c>
       <c r="E164" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="F164" t="s">
         <v>239</v>
@@ -10631,7 +10628,7 @@
         <v>25</v>
       </c>
       <c r="O164" t="s">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="P164" t="s">
         <v>79</v>
@@ -10657,7 +10654,7 @@
         <v>238</v>
       </c>
       <c r="E165" t="s">
-        <v>40</v>
+        <v>22</v>
       </c>
       <c r="F165" t="s">
         <v>239</v>
@@ -10672,22 +10669,22 @@
         <v>26</v>
       </c>
       <c r="J165" t="s">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="K165" t="s">
-        <v>86</v>
+        <v>104</v>
       </c>
       <c r="L165" t="s">
-        <v>87</v>
+        <v>105</v>
       </c>
       <c r="M165" t="s">
-        <v>88</v>
+        <v>106</v>
       </c>
       <c r="N165" t="s">
         <v>25</v>
       </c>
       <c r="O165" t="s">
-        <v>51</v>
+        <v>27</v>
       </c>
       <c r="P165" t="s">
         <v>79</v>
@@ -10743,7 +10740,7 @@
         <v>25</v>
       </c>
       <c r="O166" t="s">
-        <v>27</v>
+        <v>42</v>
       </c>
       <c r="P166" t="s">
         <v>79</v>
@@ -10799,7 +10796,7 @@
         <v>25</v>
       </c>
       <c r="O167" t="s">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="P167" t="s">
         <v>79</v>
@@ -10843,19 +10840,19 @@
         <v>51</v>
       </c>
       <c r="K168" t="s">
-        <v>104</v>
+        <v>56</v>
       </c>
       <c r="L168" t="s">
-        <v>105</v>
+        <v>114</v>
       </c>
       <c r="M168" t="s">
-        <v>106</v>
+        <v>118</v>
       </c>
       <c r="N168" t="s">
         <v>25</v>
       </c>
       <c r="O168" t="s">
-        <v>51</v>
+        <v>27</v>
       </c>
       <c r="P168" t="s">
         <v>79</v>
@@ -10911,7 +10908,7 @@
         <v>25</v>
       </c>
       <c r="O169" t="s">
-        <v>27</v>
+        <v>42</v>
       </c>
       <c r="P169" t="s">
         <v>79</v>
@@ -10937,7 +10934,7 @@
         <v>238</v>
       </c>
       <c r="E170" t="s">
-        <v>22</v>
+        <v>40</v>
       </c>
       <c r="F170" t="s">
         <v>239</v>
@@ -10967,7 +10964,7 @@
         <v>25</v>
       </c>
       <c r="O170" t="s">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="P170" t="s">
         <v>79</v>
@@ -10987,60 +10984,60 @@
         <v>19</v>
       </c>
       <c r="C171" t="s">
-        <v>35</v>
+        <v>59</v>
       </c>
       <c r="D171" t="s">
-        <v>238</v>
+        <v>21</v>
       </c>
       <c r="E171" t="s">
-        <v>40</v>
+        <v>22</v>
       </c>
       <c r="F171" t="s">
-        <v>239</v>
+        <v>267</v>
       </c>
       <c r="G171" t="s">
-        <v>77</v>
+        <v>24</v>
       </c>
       <c r="H171" t="s">
-        <v>78</v>
+        <v>25</v>
       </c>
       <c r="I171" t="s">
         <v>26</v>
       </c>
       <c r="J171" t="s">
-        <v>51</v>
+        <v>27</v>
       </c>
       <c r="K171" t="s">
-        <v>56</v>
+        <v>28</v>
       </c>
       <c r="L171" t="s">
-        <v>114</v>
+        <v>82</v>
       </c>
       <c r="M171" t="s">
-        <v>118</v>
+        <v>83</v>
       </c>
       <c r="N171" t="s">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="O171" t="s">
-        <v>51</v>
+        <v>25</v>
       </c>
       <c r="P171" t="s">
         <v>79</v>
       </c>
       <c r="Q171" t="s">
-        <v>240</v>
+        <v>25</v>
       </c>
       <c r="R171" t="s">
-        <v>25</v>
+        <v>33</v>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="B172" t="s">
-        <v>19</v>
+        <v>35</v>
       </c>
       <c r="C172" t="s">
         <v>59</v>
@@ -11052,7 +11049,7 @@
         <v>22</v>
       </c>
       <c r="F172" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="G172" t="s">
         <v>24</v>
@@ -11096,19 +11093,19 @@
         <v>269</v>
       </c>
       <c r="B173" t="s">
-        <v>35</v>
+        <v>19</v>
       </c>
       <c r="C173" t="s">
         <v>59</v>
       </c>
       <c r="D173" t="s">
-        <v>21</v>
+        <v>270</v>
       </c>
       <c r="E173" t="s">
-        <v>22</v>
+        <v>40</v>
       </c>
       <c r="F173" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="G173" t="s">
         <v>24</v>
@@ -11120,25 +11117,25 @@
         <v>26</v>
       </c>
       <c r="J173" t="s">
-        <v>27</v>
+        <v>42</v>
       </c>
       <c r="K173" t="s">
-        <v>28</v>
+        <v>86</v>
       </c>
       <c r="L173" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="M173" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="N173" t="s">
-        <v>31</v>
+        <v>271</v>
       </c>
       <c r="O173" t="s">
         <v>25</v>
       </c>
       <c r="P173" t="s">
-        <v>79</v>
+        <v>272</v>
       </c>
       <c r="Q173" t="s">
         <v>25</v>
@@ -11149,22 +11146,22 @@
     </row>
     <row r="174">
       <c r="A174" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
       <c r="B174" t="s">
-        <v>19</v>
+        <v>35</v>
       </c>
       <c r="C174" t="s">
         <v>59</v>
       </c>
       <c r="D174" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="E174" t="s">
         <v>40</v>
       </c>
       <c r="F174" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="G174" t="s">
         <v>24</v>
@@ -11188,13 +11185,13 @@
         <v>88</v>
       </c>
       <c r="N174" t="s">
+        <v>271</v>
+      </c>
+      <c r="O174" t="s">
+        <v>25</v>
+      </c>
+      <c r="P174" t="s">
         <v>272</v>
-      </c>
-      <c r="O174" t="s">
-        <v>25</v>
-      </c>
-      <c r="P174" t="s">
-        <v>273</v>
       </c>
       <c r="Q174" t="s">
         <v>25</v>
@@ -11208,19 +11205,19 @@
         <v>274</v>
       </c>
       <c r="B175" t="s">
-        <v>35</v>
+        <v>19</v>
       </c>
       <c r="C175" t="s">
         <v>59</v>
       </c>
       <c r="D175" t="s">
-        <v>271</v>
+        <v>21</v>
       </c>
       <c r="E175" t="s">
-        <v>40</v>
+        <v>22</v>
       </c>
       <c r="F175" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="G175" t="s">
         <v>24</v>
@@ -11238,19 +11235,19 @@
         <v>86</v>
       </c>
       <c r="L175" t="s">
-        <v>87</v>
+        <v>96</v>
       </c>
       <c r="M175" t="s">
-        <v>88</v>
+        <v>97</v>
       </c>
       <c r="N175" t="s">
-        <v>272</v>
+        <v>31</v>
       </c>
       <c r="O175" t="s">
         <v>25</v>
       </c>
       <c r="P175" t="s">
-        <v>273</v>
+        <v>79</v>
       </c>
       <c r="Q175" t="s">
         <v>25</v>
@@ -11264,7 +11261,7 @@
         <v>275</v>
       </c>
       <c r="B176" t="s">
-        <v>19</v>
+        <v>35</v>
       </c>
       <c r="C176" t="s">
         <v>59</v>
@@ -11276,7 +11273,7 @@
         <v>22</v>
       </c>
       <c r="F176" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="G176" t="s">
         <v>24</v>
@@ -11320,7 +11317,7 @@
         <v>276</v>
       </c>
       <c r="B177" t="s">
-        <v>35</v>
+        <v>19</v>
       </c>
       <c r="C177" t="s">
         <v>59</v>
@@ -11329,10 +11326,10 @@
         <v>21</v>
       </c>
       <c r="E177" t="s">
-        <v>22</v>
+        <v>35</v>
       </c>
       <c r="F177" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="G177" t="s">
         <v>24</v>
@@ -11347,13 +11344,13 @@
         <v>42</v>
       </c>
       <c r="K177" t="s">
-        <v>86</v>
+        <v>100</v>
       </c>
       <c r="L177" t="s">
         <v>96</v>
       </c>
       <c r="M177" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="N177" t="s">
         <v>31</v>
@@ -11362,7 +11359,7 @@
         <v>25</v>
       </c>
       <c r="P177" t="s">
-        <v>79</v>
+        <v>93</v>
       </c>
       <c r="Q177" t="s">
         <v>25</v>
@@ -11376,7 +11373,7 @@
         <v>277</v>
       </c>
       <c r="B178" t="s">
-        <v>19</v>
+        <v>35</v>
       </c>
       <c r="C178" t="s">
         <v>59</v>
@@ -11388,7 +11385,7 @@
         <v>35</v>
       </c>
       <c r="F178" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="G178" t="s">
         <v>24</v>
@@ -11432,7 +11429,7 @@
         <v>278</v>
       </c>
       <c r="B179" t="s">
-        <v>35</v>
+        <v>19</v>
       </c>
       <c r="C179" t="s">
         <v>59</v>
@@ -11441,10 +11438,10 @@
         <v>21</v>
       </c>
       <c r="E179" t="s">
-        <v>35</v>
+        <v>22</v>
       </c>
       <c r="F179" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="G179" t="s">
         <v>24</v>
@@ -11456,16 +11453,16 @@
         <v>26</v>
       </c>
       <c r="J179" t="s">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="K179" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="L179" t="s">
-        <v>96</v>
+        <v>105</v>
       </c>
       <c r="M179" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="N179" t="s">
         <v>31</v>
@@ -11474,7 +11471,7 @@
         <v>25</v>
       </c>
       <c r="P179" t="s">
-        <v>93</v>
+        <v>79</v>
       </c>
       <c r="Q179" t="s">
         <v>25</v>
@@ -11488,7 +11485,7 @@
         <v>279</v>
       </c>
       <c r="B180" t="s">
-        <v>19</v>
+        <v>35</v>
       </c>
       <c r="C180" t="s">
         <v>59</v>
@@ -11500,7 +11497,7 @@
         <v>22</v>
       </c>
       <c r="F180" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="G180" t="s">
         <v>24</v>
@@ -11544,7 +11541,7 @@
         <v>280</v>
       </c>
       <c r="B181" t="s">
-        <v>35</v>
+        <v>19</v>
       </c>
       <c r="C181" t="s">
         <v>59</v>
@@ -11556,7 +11553,7 @@
         <v>22</v>
       </c>
       <c r="F181" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="G181" t="s">
         <v>24</v>
@@ -11571,13 +11568,13 @@
         <v>51</v>
       </c>
       <c r="K181" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="L181" t="s">
         <v>105</v>
       </c>
       <c r="M181" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="N181" t="s">
         <v>31</v>
@@ -11586,7 +11583,7 @@
         <v>25</v>
       </c>
       <c r="P181" t="s">
-        <v>79</v>
+        <v>93</v>
       </c>
       <c r="Q181" t="s">
         <v>25</v>
@@ -11600,7 +11597,7 @@
         <v>281</v>
       </c>
       <c r="B182" t="s">
-        <v>19</v>
+        <v>35</v>
       </c>
       <c r="C182" t="s">
         <v>59</v>
@@ -11612,7 +11609,7 @@
         <v>22</v>
       </c>
       <c r="F182" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="G182" t="s">
         <v>24</v>
@@ -11656,7 +11653,7 @@
         <v>282</v>
       </c>
       <c r="B183" t="s">
-        <v>35</v>
+        <v>19</v>
       </c>
       <c r="C183" t="s">
         <v>59</v>
@@ -11668,7 +11665,7 @@
         <v>22</v>
       </c>
       <c r="F183" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="G183" t="s">
         <v>24</v>
@@ -11683,13 +11680,13 @@
         <v>51</v>
       </c>
       <c r="K183" t="s">
-        <v>109</v>
+        <v>56</v>
       </c>
       <c r="L183" t="s">
-        <v>105</v>
+        <v>114</v>
       </c>
       <c r="M183" t="s">
-        <v>110</v>
+        <v>118</v>
       </c>
       <c r="N183" t="s">
         <v>31</v>
@@ -11698,7 +11695,7 @@
         <v>25</v>
       </c>
       <c r="P183" t="s">
-        <v>93</v>
+        <v>79</v>
       </c>
       <c r="Q183" t="s">
         <v>25</v>
@@ -11712,7 +11709,7 @@
         <v>283</v>
       </c>
       <c r="B184" t="s">
-        <v>19</v>
+        <v>35</v>
       </c>
       <c r="C184" t="s">
         <v>59</v>
@@ -11724,7 +11721,7 @@
         <v>22</v>
       </c>
       <c r="F184" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="G184" t="s">
         <v>24</v>
@@ -11768,7 +11765,7 @@
         <v>284</v>
       </c>
       <c r="B185" t="s">
-        <v>35</v>
+        <v>19</v>
       </c>
       <c r="C185" t="s">
         <v>59</v>
@@ -11780,7 +11777,7 @@
         <v>22</v>
       </c>
       <c r="F185" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="G185" t="s">
         <v>24</v>
@@ -11792,16 +11789,16 @@
         <v>26</v>
       </c>
       <c r="J185" t="s">
-        <v>51</v>
+        <v>27</v>
       </c>
       <c r="K185" t="s">
-        <v>56</v>
+        <v>28</v>
       </c>
       <c r="L185" t="s">
-        <v>114</v>
+        <v>82</v>
       </c>
       <c r="M185" t="s">
-        <v>118</v>
+        <v>83</v>
       </c>
       <c r="N185" t="s">
         <v>31</v>
@@ -11824,7 +11821,7 @@
         <v>285</v>
       </c>
       <c r="B186" t="s">
-        <v>19</v>
+        <v>35</v>
       </c>
       <c r="C186" t="s">
         <v>59</v>
@@ -11836,7 +11833,7 @@
         <v>22</v>
       </c>
       <c r="F186" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="G186" t="s">
         <v>24</v>
@@ -11880,19 +11877,19 @@
         <v>286</v>
       </c>
       <c r="B187" t="s">
-        <v>35</v>
+        <v>19</v>
       </c>
       <c r="C187" t="s">
         <v>59</v>
       </c>
       <c r="D187" t="s">
-        <v>21</v>
+        <v>270</v>
       </c>
       <c r="E187" t="s">
         <v>22</v>
       </c>
       <c r="F187" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="G187" t="s">
         <v>24</v>
@@ -11904,25 +11901,25 @@
         <v>26</v>
       </c>
       <c r="J187" t="s">
-        <v>27</v>
+        <v>42</v>
       </c>
       <c r="K187" t="s">
-        <v>28</v>
+        <v>86</v>
       </c>
       <c r="L187" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="M187" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="N187" t="s">
-        <v>31</v>
+        <v>271</v>
       </c>
       <c r="O187" t="s">
         <v>25</v>
       </c>
       <c r="P187" t="s">
-        <v>79</v>
+        <v>272</v>
       </c>
       <c r="Q187" t="s">
         <v>25</v>
@@ -11936,19 +11933,19 @@
         <v>287</v>
       </c>
       <c r="B188" t="s">
-        <v>19</v>
+        <v>35</v>
       </c>
       <c r="C188" t="s">
         <v>59</v>
       </c>
       <c r="D188" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="E188" t="s">
         <v>22</v>
       </c>
       <c r="F188" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="G188" t="s">
         <v>24</v>
@@ -11972,13 +11969,13 @@
         <v>88</v>
       </c>
       <c r="N188" t="s">
+        <v>271</v>
+      </c>
+      <c r="O188" t="s">
+        <v>25</v>
+      </c>
+      <c r="P188" t="s">
         <v>272</v>
-      </c>
-      <c r="O188" t="s">
-        <v>25</v>
-      </c>
-      <c r="P188" t="s">
-        <v>273</v>
       </c>
       <c r="Q188" t="s">
         <v>25</v>
@@ -11992,19 +11989,19 @@
         <v>288</v>
       </c>
       <c r="B189" t="s">
-        <v>35</v>
+        <v>19</v>
       </c>
       <c r="C189" t="s">
         <v>59</v>
       </c>
       <c r="D189" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="E189" t="s">
         <v>22</v>
       </c>
       <c r="F189" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="G189" t="s">
         <v>24</v>
@@ -12019,22 +12016,22 @@
         <v>42</v>
       </c>
       <c r="K189" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="L189" t="s">
         <v>87</v>
       </c>
       <c r="M189" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="N189" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="O189" t="s">
         <v>25</v>
       </c>
       <c r="P189" t="s">
-        <v>273</v>
+        <v>289</v>
       </c>
       <c r="Q189" t="s">
         <v>25</v>
@@ -12045,22 +12042,22 @@
     </row>
     <row r="190">
       <c r="A190" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="B190" t="s">
-        <v>19</v>
+        <v>35</v>
       </c>
       <c r="C190" t="s">
         <v>59</v>
       </c>
       <c r="D190" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="E190" t="s">
         <v>22</v>
       </c>
       <c r="F190" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="G190" t="s">
         <v>24</v>
@@ -12084,13 +12081,13 @@
         <v>92</v>
       </c>
       <c r="N190" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="O190" t="s">
         <v>25</v>
       </c>
       <c r="P190" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="Q190" t="s">
         <v>25</v>
@@ -12104,19 +12101,19 @@
         <v>291</v>
       </c>
       <c r="B191" t="s">
-        <v>35</v>
+        <v>19</v>
       </c>
       <c r="C191" t="s">
         <v>59</v>
       </c>
       <c r="D191" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="E191" t="s">
         <v>22</v>
       </c>
       <c r="F191" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="G191" t="s">
         <v>24</v>
@@ -12131,22 +12128,22 @@
         <v>42</v>
       </c>
       <c r="K191" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="L191" t="s">
-        <v>87</v>
+        <v>96</v>
       </c>
       <c r="M191" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="N191" t="s">
+        <v>271</v>
+      </c>
+      <c r="O191" t="s">
+        <v>25</v>
+      </c>
+      <c r="P191" t="s">
         <v>272</v>
-      </c>
-      <c r="O191" t="s">
-        <v>25</v>
-      </c>
-      <c r="P191" t="s">
-        <v>290</v>
       </c>
       <c r="Q191" t="s">
         <v>25</v>
@@ -12160,19 +12157,19 @@
         <v>292</v>
       </c>
       <c r="B192" t="s">
-        <v>19</v>
+        <v>35</v>
       </c>
       <c r="C192" t="s">
         <v>59</v>
       </c>
       <c r="D192" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="E192" t="s">
         <v>22</v>
       </c>
       <c r="F192" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="G192" t="s">
         <v>24</v>
@@ -12196,13 +12193,13 @@
         <v>97</v>
       </c>
       <c r="N192" t="s">
+        <v>271</v>
+      </c>
+      <c r="O192" t="s">
+        <v>25</v>
+      </c>
+      <c r="P192" t="s">
         <v>272</v>
-      </c>
-      <c r="O192" t="s">
-        <v>25</v>
-      </c>
-      <c r="P192" t="s">
-        <v>273</v>
       </c>
       <c r="Q192" t="s">
         <v>25</v>
@@ -12216,19 +12213,19 @@
         <v>293</v>
       </c>
       <c r="B193" t="s">
-        <v>35</v>
+        <v>19</v>
       </c>
       <c r="C193" t="s">
         <v>59</v>
       </c>
       <c r="D193" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="E193" t="s">
-        <v>22</v>
+        <v>59</v>
       </c>
       <c r="F193" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="G193" t="s">
         <v>24</v>
@@ -12243,22 +12240,22 @@
         <v>42</v>
       </c>
       <c r="K193" t="s">
-        <v>86</v>
+        <v>100</v>
       </c>
       <c r="L193" t="s">
         <v>96</v>
       </c>
       <c r="M193" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="N193" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="O193" t="s">
         <v>25</v>
       </c>
       <c r="P193" t="s">
-        <v>273</v>
+        <v>289</v>
       </c>
       <c r="Q193" t="s">
         <v>25</v>
@@ -12272,19 +12269,19 @@
         <v>294</v>
       </c>
       <c r="B194" t="s">
-        <v>19</v>
+        <v>35</v>
       </c>
       <c r="C194" t="s">
         <v>59</v>
       </c>
       <c r="D194" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="E194" t="s">
         <v>59</v>
       </c>
       <c r="F194" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="G194" t="s">
         <v>24</v>
@@ -12308,13 +12305,13 @@
         <v>101</v>
       </c>
       <c r="N194" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="O194" t="s">
         <v>25</v>
       </c>
       <c r="P194" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="Q194" t="s">
         <v>25</v>
@@ -12328,19 +12325,19 @@
         <v>295</v>
       </c>
       <c r="B195" t="s">
-        <v>35</v>
+        <v>19</v>
       </c>
       <c r="C195" t="s">
         <v>59</v>
       </c>
       <c r="D195" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="E195" t="s">
-        <v>59</v>
+        <v>40</v>
       </c>
       <c r="F195" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="G195" t="s">
         <v>24</v>
@@ -12352,25 +12349,25 @@
         <v>26</v>
       </c>
       <c r="J195" t="s">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="K195" t="s">
-        <v>100</v>
+        <v>109</v>
       </c>
       <c r="L195" t="s">
-        <v>96</v>
+        <v>105</v>
       </c>
       <c r="M195" t="s">
-        <v>101</v>
+        <v>110</v>
       </c>
       <c r="N195" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="O195" t="s">
         <v>25</v>
       </c>
       <c r="P195" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="Q195" t="s">
         <v>25</v>
@@ -12384,19 +12381,19 @@
         <v>296</v>
       </c>
       <c r="B196" t="s">
-        <v>19</v>
+        <v>35</v>
       </c>
       <c r="C196" t="s">
         <v>59</v>
       </c>
       <c r="D196" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="E196" t="s">
         <v>40</v>
       </c>
       <c r="F196" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="G196" t="s">
         <v>24</v>
@@ -12420,13 +12417,13 @@
         <v>110</v>
       </c>
       <c r="N196" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="O196" t="s">
         <v>25</v>
       </c>
       <c r="P196" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="Q196" t="s">
         <v>25</v>
@@ -12440,19 +12437,19 @@
         <v>297</v>
       </c>
       <c r="B197" t="s">
-        <v>35</v>
+        <v>19</v>
       </c>
       <c r="C197" t="s">
         <v>59</v>
       </c>
       <c r="D197" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="E197" t="s">
         <v>40</v>
       </c>
       <c r="F197" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="G197" t="s">
         <v>24</v>
@@ -12467,22 +12464,22 @@
         <v>51</v>
       </c>
       <c r="K197" t="s">
-        <v>109</v>
+        <v>56</v>
       </c>
       <c r="L197" t="s">
-        <v>105</v>
+        <v>114</v>
       </c>
       <c r="M197" t="s">
-        <v>110</v>
+        <v>118</v>
       </c>
       <c r="N197" t="s">
+        <v>271</v>
+      </c>
+      <c r="O197" t="s">
+        <v>25</v>
+      </c>
+      <c r="P197" t="s">
         <v>272</v>
-      </c>
-      <c r="O197" t="s">
-        <v>25</v>
-      </c>
-      <c r="P197" t="s">
-        <v>290</v>
       </c>
       <c r="Q197" t="s">
         <v>25</v>
@@ -12496,19 +12493,19 @@
         <v>298</v>
       </c>
       <c r="B198" t="s">
-        <v>19</v>
+        <v>35</v>
       </c>
       <c r="C198" t="s">
         <v>59</v>
       </c>
       <c r="D198" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="E198" t="s">
         <v>40</v>
       </c>
       <c r="F198" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="G198" t="s">
         <v>24</v>
@@ -12532,13 +12529,13 @@
         <v>118</v>
       </c>
       <c r="N198" t="s">
+        <v>271</v>
+      </c>
+      <c r="O198" t="s">
+        <v>25</v>
+      </c>
+      <c r="P198" t="s">
         <v>272</v>
-      </c>
-      <c r="O198" t="s">
-        <v>25</v>
-      </c>
-      <c r="P198" t="s">
-        <v>273</v>
       </c>
       <c r="Q198" t="s">
         <v>25</v>
@@ -12552,19 +12549,19 @@
         <v>299</v>
       </c>
       <c r="B199" t="s">
-        <v>35</v>
+        <v>19</v>
       </c>
       <c r="C199" t="s">
         <v>59</v>
       </c>
       <c r="D199" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="E199" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="F199" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="G199" t="s">
         <v>24</v>
@@ -12579,22 +12576,22 @@
         <v>51</v>
       </c>
       <c r="K199" t="s">
-        <v>56</v>
+        <v>104</v>
       </c>
       <c r="L199" t="s">
-        <v>114</v>
+        <v>105</v>
       </c>
       <c r="M199" t="s">
-        <v>118</v>
+        <v>106</v>
       </c>
       <c r="N199" t="s">
+        <v>271</v>
+      </c>
+      <c r="O199" t="s">
+        <v>25</v>
+      </c>
+      <c r="P199" t="s">
         <v>272</v>
-      </c>
-      <c r="O199" t="s">
-        <v>25</v>
-      </c>
-      <c r="P199" t="s">
-        <v>273</v>
       </c>
       <c r="Q199" t="s">
         <v>25</v>
@@ -12608,19 +12605,19 @@
         <v>300</v>
       </c>
       <c r="B200" t="s">
-        <v>19</v>
+        <v>35</v>
       </c>
       <c r="C200" t="s">
         <v>59</v>
       </c>
       <c r="D200" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="E200" t="s">
         <v>35</v>
       </c>
       <c r="F200" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="G200" t="s">
         <v>24</v>
@@ -12644,13 +12641,13 @@
         <v>106</v>
       </c>
       <c r="N200" t="s">
+        <v>271</v>
+      </c>
+      <c r="O200" t="s">
+        <v>25</v>
+      </c>
+      <c r="P200" t="s">
         <v>272</v>
-      </c>
-      <c r="O200" t="s">
-        <v>25</v>
-      </c>
-      <c r="P200" t="s">
-        <v>273</v>
       </c>
       <c r="Q200" t="s">
         <v>25</v>
@@ -12664,22 +12661,22 @@
         <v>301</v>
       </c>
       <c r="B201" t="s">
-        <v>35</v>
+        <v>19</v>
       </c>
       <c r="C201" t="s">
         <v>59</v>
       </c>
       <c r="D201" t="s">
-        <v>271</v>
+        <v>302</v>
       </c>
       <c r="E201" t="s">
-        <v>35</v>
+        <v>22</v>
       </c>
       <c r="F201" t="s">
-        <v>268</v>
+        <v>182</v>
       </c>
       <c r="G201" t="s">
-        <v>24</v>
+        <v>77</v>
       </c>
       <c r="H201" t="s">
         <v>25</v>
@@ -12688,36 +12685,36 @@
         <v>26</v>
       </c>
       <c r="J201" t="s">
-        <v>51</v>
+        <v>42</v>
       </c>
       <c r="K201" t="s">
-        <v>104</v>
+        <v>86</v>
       </c>
       <c r="L201" t="s">
-        <v>105</v>
+        <v>87</v>
       </c>
       <c r="M201" t="s">
-        <v>106</v>
+        <v>88</v>
       </c>
       <c r="N201" t="s">
-        <v>272</v>
+        <v>25</v>
       </c>
       <c r="O201" t="s">
         <v>25</v>
       </c>
       <c r="P201" t="s">
-        <v>273</v>
+        <v>303</v>
       </c>
       <c r="Q201" t="s">
-        <v>25</v>
+        <v>183</v>
       </c>
       <c r="R201" t="s">
-        <v>33</v>
+        <v>183</v>
       </c>
     </row>
     <row r="202">
       <c r="A202" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="B202" t="s">
         <v>19</v>
@@ -12726,7 +12723,7 @@
         <v>59</v>
       </c>
       <c r="D202" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="E202" t="s">
         <v>22</v>
@@ -12747,13 +12744,13 @@
         <v>42</v>
       </c>
       <c r="K202" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="L202" t="s">
         <v>87</v>
       </c>
       <c r="M202" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="N202" t="s">
         <v>25</v>
@@ -12762,7 +12759,7 @@
         <v>25</v>
       </c>
       <c r="P202" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="Q202" t="s">
         <v>183</v>
@@ -12773,16 +12770,16 @@
     </row>
     <row r="203">
       <c r="A203" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="B203" t="s">
-        <v>19</v>
+        <v>35</v>
       </c>
       <c r="C203" t="s">
         <v>59</v>
       </c>
       <c r="D203" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="E203" t="s">
         <v>22</v>
@@ -12818,7 +12815,7 @@
         <v>25</v>
       </c>
       <c r="P203" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="Q203" t="s">
         <v>183</v>
@@ -12832,16 +12829,16 @@
         <v>307</v>
       </c>
       <c r="B204" t="s">
-        <v>35</v>
+        <v>19</v>
       </c>
       <c r="C204" t="s">
         <v>59</v>
       </c>
       <c r="D204" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="E204" t="s">
-        <v>22</v>
+        <v>35</v>
       </c>
       <c r="F204" t="s">
         <v>182</v>
@@ -12859,13 +12856,13 @@
         <v>42</v>
       </c>
       <c r="K204" t="s">
-        <v>91</v>
+        <v>100</v>
       </c>
       <c r="L204" t="s">
-        <v>87</v>
+        <v>96</v>
       </c>
       <c r="M204" t="s">
-        <v>92</v>
+        <v>101</v>
       </c>
       <c r="N204" t="s">
         <v>25</v>
@@ -12874,7 +12871,7 @@
         <v>25</v>
       </c>
       <c r="P204" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="Q204" t="s">
         <v>183</v>
@@ -12888,13 +12885,13 @@
         <v>308</v>
       </c>
       <c r="B205" t="s">
-        <v>19</v>
+        <v>35</v>
       </c>
       <c r="C205" t="s">
         <v>59</v>
       </c>
       <c r="D205" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="E205" t="s">
         <v>35</v>
@@ -12930,7 +12927,7 @@
         <v>25</v>
       </c>
       <c r="P205" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="Q205" t="s">
         <v>183</v>
@@ -12944,13 +12941,13 @@
         <v>309</v>
       </c>
       <c r="B206" t="s">
-        <v>35</v>
+        <v>19</v>
       </c>
       <c r="C206" t="s">
         <v>59</v>
       </c>
       <c r="D206" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="E206" t="s">
         <v>35</v>
@@ -12968,16 +12965,16 @@
         <v>26</v>
       </c>
       <c r="J206" t="s">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="K206" t="s">
-        <v>100</v>
+        <v>56</v>
       </c>
       <c r="L206" t="s">
-        <v>96</v>
+        <v>114</v>
       </c>
       <c r="M206" t="s">
-        <v>101</v>
+        <v>118</v>
       </c>
       <c r="N206" t="s">
         <v>25</v>
@@ -12986,7 +12983,7 @@
         <v>25</v>
       </c>
       <c r="P206" t="s">
-        <v>306</v>
+        <v>303</v>
       </c>
       <c r="Q206" t="s">
         <v>183</v>
@@ -13006,13 +13003,13 @@
         <v>59</v>
       </c>
       <c r="D207" t="s">
-        <v>303</v>
+        <v>311</v>
       </c>
       <c r="E207" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="F207" t="s">
-        <v>182</v>
+        <v>210</v>
       </c>
       <c r="G207" t="s">
         <v>77</v>
@@ -13024,16 +13021,16 @@
         <v>26</v>
       </c>
       <c r="J207" t="s">
-        <v>51</v>
+        <v>42</v>
       </c>
       <c r="K207" t="s">
-        <v>56</v>
+        <v>86</v>
       </c>
       <c r="L207" t="s">
-        <v>114</v>
+        <v>96</v>
       </c>
       <c r="M207" t="s">
-        <v>118</v>
+        <v>97</v>
       </c>
       <c r="N207" t="s">
         <v>25</v>
@@ -13042,18 +13039,18 @@
         <v>25</v>
       </c>
       <c r="P207" t="s">
-        <v>304</v>
+        <v>312</v>
       </c>
       <c r="Q207" t="s">
-        <v>183</v>
+        <v>211</v>
       </c>
       <c r="R207" t="s">
-        <v>183</v>
+        <v>25</v>
       </c>
     </row>
     <row r="208">
       <c r="A208" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="B208" t="s">
         <v>19</v>
@@ -13062,10 +13059,10 @@
         <v>59</v>
       </c>
       <c r="D208" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="E208" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="F208" t="s">
         <v>210</v>
@@ -13083,13 +13080,13 @@
         <v>42</v>
       </c>
       <c r="K208" t="s">
-        <v>86</v>
+        <v>100</v>
       </c>
       <c r="L208" t="s">
         <v>96</v>
       </c>
       <c r="M208" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="N208" t="s">
         <v>25</v>
@@ -13098,7 +13095,7 @@
         <v>25</v>
       </c>
       <c r="P208" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="Q208" t="s">
         <v>211</v>
@@ -13109,7 +13106,7 @@
     </row>
     <row r="209">
       <c r="A209" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="B209" t="s">
         <v>19</v>
@@ -13118,10 +13115,10 @@
         <v>59</v>
       </c>
       <c r="D209" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="E209" t="s">
-        <v>35</v>
+        <v>22</v>
       </c>
       <c r="F209" t="s">
         <v>210</v>
@@ -13139,13 +13136,13 @@
         <v>42</v>
       </c>
       <c r="K209" t="s">
-        <v>100</v>
+        <v>86</v>
       </c>
       <c r="L209" t="s">
-        <v>96</v>
+        <v>87</v>
       </c>
       <c r="M209" t="s">
-        <v>101</v>
+        <v>88</v>
       </c>
       <c r="N209" t="s">
         <v>25</v>
@@ -13154,7 +13151,7 @@
         <v>25</v>
       </c>
       <c r="P209" t="s">
-        <v>315</v>
+        <v>312</v>
       </c>
       <c r="Q209" t="s">
         <v>211</v>
@@ -13168,13 +13165,13 @@
         <v>316</v>
       </c>
       <c r="B210" t="s">
-        <v>19</v>
+        <v>35</v>
       </c>
       <c r="C210" t="s">
         <v>59</v>
       </c>
       <c r="D210" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="E210" t="s">
         <v>22</v>
@@ -13210,7 +13207,7 @@
         <v>25</v>
       </c>
       <c r="P210" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="Q210" t="s">
         <v>211</v>
@@ -13224,13 +13221,13 @@
         <v>317</v>
       </c>
       <c r="B211" t="s">
-        <v>35</v>
+        <v>19</v>
       </c>
       <c r="C211" t="s">
         <v>59</v>
       </c>
       <c r="D211" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="E211" t="s">
         <v>22</v>
@@ -13251,13 +13248,13 @@
         <v>42</v>
       </c>
       <c r="K211" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="L211" t="s">
         <v>87</v>
       </c>
       <c r="M211" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="N211" t="s">
         <v>25</v>
@@ -13266,7 +13263,7 @@
         <v>25</v>
       </c>
       <c r="P211" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="Q211" t="s">
         <v>211</v>
@@ -13280,13 +13277,13 @@
         <v>318</v>
       </c>
       <c r="B212" t="s">
-        <v>19</v>
+        <v>35</v>
       </c>
       <c r="C212" t="s">
         <v>59</v>
       </c>
       <c r="D212" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="E212" t="s">
         <v>22</v>
@@ -13322,7 +13319,7 @@
         <v>25</v>
       </c>
       <c r="P212" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="Q212" t="s">
         <v>211</v>
@@ -13336,16 +13333,16 @@
         <v>319</v>
       </c>
       <c r="B213" t="s">
-        <v>35</v>
+        <v>19</v>
       </c>
       <c r="C213" t="s">
         <v>59</v>
       </c>
       <c r="D213" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="E213" t="s">
-        <v>22</v>
+        <v>59</v>
       </c>
       <c r="F213" t="s">
         <v>210</v>
@@ -13360,16 +13357,16 @@
         <v>26</v>
       </c>
       <c r="J213" t="s">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="K213" t="s">
-        <v>91</v>
+        <v>109</v>
       </c>
       <c r="L213" t="s">
-        <v>87</v>
+        <v>105</v>
       </c>
       <c r="M213" t="s">
-        <v>92</v>
+        <v>110</v>
       </c>
       <c r="N213" t="s">
         <v>25</v>
@@ -13378,7 +13375,7 @@
         <v>25</v>
       </c>
       <c r="P213" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="Q213" t="s">
         <v>211</v>
@@ -13392,13 +13389,13 @@
         <v>320</v>
       </c>
       <c r="B214" t="s">
-        <v>19</v>
+        <v>35</v>
       </c>
       <c r="C214" t="s">
         <v>59</v>
       </c>
       <c r="D214" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="E214" t="s">
         <v>59</v>
@@ -13434,7 +13431,7 @@
         <v>25</v>
       </c>
       <c r="P214" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="Q214" t="s">
         <v>211</v>
@@ -13448,13 +13445,13 @@
         <v>321</v>
       </c>
       <c r="B215" t="s">
-        <v>35</v>
+        <v>19</v>
       </c>
       <c r="C215" t="s">
         <v>59</v>
       </c>
       <c r="D215" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="E215" t="s">
         <v>59</v>
@@ -13475,13 +13472,13 @@
         <v>51</v>
       </c>
       <c r="K215" t="s">
-        <v>109</v>
+        <v>56</v>
       </c>
       <c r="L215" t="s">
-        <v>105</v>
+        <v>114</v>
       </c>
       <c r="M215" t="s">
-        <v>110</v>
+        <v>118</v>
       </c>
       <c r="N215" t="s">
         <v>25</v>
@@ -13490,7 +13487,7 @@
         <v>25</v>
       </c>
       <c r="P215" t="s">
-        <v>315</v>
+        <v>312</v>
       </c>
       <c r="Q215" t="s">
         <v>211</v>
@@ -13504,16 +13501,16 @@
         <v>322</v>
       </c>
       <c r="B216" t="s">
-        <v>19</v>
+        <v>35</v>
       </c>
       <c r="C216" t="s">
         <v>59</v>
       </c>
       <c r="D216" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="E216" t="s">
-        <v>59</v>
+        <v>35</v>
       </c>
       <c r="F216" t="s">
         <v>210</v>
@@ -13546,7 +13543,7 @@
         <v>25</v>
       </c>
       <c r="P216" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="Q216" t="s">
         <v>211</v>
@@ -13560,52 +13557,52 @@
         <v>323</v>
       </c>
       <c r="B217" t="s">
-        <v>35</v>
+        <v>19</v>
       </c>
       <c r="C217" t="s">
+        <v>35</v>
+      </c>
+      <c r="D217" t="s">
+        <v>324</v>
+      </c>
+      <c r="E217" t="s">
         <v>59</v>
       </c>
-      <c r="D217" t="s">
-        <v>312</v>
-      </c>
-      <c r="E217" t="s">
-        <v>35</v>
-      </c>
       <c r="F217" t="s">
-        <v>210</v>
+        <v>325</v>
       </c>
       <c r="G217" t="s">
-        <v>77</v>
+        <v>24</v>
       </c>
       <c r="H217" t="s">
-        <v>25</v>
+        <v>123</v>
       </c>
       <c r="I217" t="s">
         <v>26</v>
       </c>
       <c r="J217" t="s">
-        <v>51</v>
+        <v>27</v>
       </c>
       <c r="K217" t="s">
-        <v>56</v>
+        <v>28</v>
       </c>
       <c r="L217" t="s">
-        <v>114</v>
+        <v>82</v>
       </c>
       <c r="M217" t="s">
-        <v>118</v>
+        <v>83</v>
       </c>
       <c r="N217" t="s">
         <v>25</v>
       </c>
       <c r="O217" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="P217" t="s">
-        <v>313</v>
+        <v>79</v>
       </c>
       <c r="Q217" t="s">
-        <v>211</v>
+        <v>325</v>
       </c>
       <c r="R217" t="s">
         <v>25</v>
@@ -13613,22 +13610,22 @@
     </row>
     <row r="218">
       <c r="A218" t="s">
+        <v>326</v>
+      </c>
+      <c r="B218" t="s">
+        <v>19</v>
+      </c>
+      <c r="C218" t="s">
+        <v>35</v>
+      </c>
+      <c r="D218" t="s">
         <v>324</v>
-      </c>
-      <c r="B218" t="s">
-        <v>19</v>
-      </c>
-      <c r="C218" t="s">
-        <v>35</v>
-      </c>
-      <c r="D218" t="s">
-        <v>325</v>
       </c>
       <c r="E218" t="s">
         <v>59</v>
       </c>
       <c r="F218" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="G218" t="s">
         <v>24</v>
@@ -13655,13 +13652,13 @@
         <v>25</v>
       </c>
       <c r="O218" t="s">
-        <v>27</v>
+        <v>42</v>
       </c>
       <c r="P218" t="s">
         <v>79</v>
       </c>
       <c r="Q218" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="R218" t="s">
         <v>25</v>
@@ -13678,13 +13675,13 @@
         <v>35</v>
       </c>
       <c r="D219" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="E219" t="s">
         <v>59</v>
       </c>
       <c r="F219" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="G219" t="s">
         <v>24</v>
@@ -13711,13 +13708,13 @@
         <v>25</v>
       </c>
       <c r="O219" t="s">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="P219" t="s">
         <v>79</v>
       </c>
       <c r="Q219" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="R219" t="s">
         <v>25</v>
@@ -13734,13 +13731,13 @@
         <v>35</v>
       </c>
       <c r="D220" t="s">
+        <v>324</v>
+      </c>
+      <c r="E220" t="s">
+        <v>40</v>
+      </c>
+      <c r="F220" t="s">
         <v>325</v>
-      </c>
-      <c r="E220" t="s">
-        <v>59</v>
-      </c>
-      <c r="F220" t="s">
-        <v>326</v>
       </c>
       <c r="G220" t="s">
         <v>24</v>
@@ -13752,28 +13749,28 @@
         <v>26</v>
       </c>
       <c r="J220" t="s">
+        <v>42</v>
+      </c>
+      <c r="K220" t="s">
+        <v>86</v>
+      </c>
+      <c r="L220" t="s">
+        <v>96</v>
+      </c>
+      <c r="M220" t="s">
+        <v>97</v>
+      </c>
+      <c r="N220" t="s">
+        <v>25</v>
+      </c>
+      <c r="O220" t="s">
         <v>27</v>
       </c>
-      <c r="K220" t="s">
-        <v>28</v>
-      </c>
-      <c r="L220" t="s">
-        <v>82</v>
-      </c>
-      <c r="M220" t="s">
-        <v>83</v>
-      </c>
-      <c r="N220" t="s">
-        <v>25</v>
-      </c>
-      <c r="O220" t="s">
-        <v>51</v>
-      </c>
       <c r="P220" t="s">
         <v>79</v>
       </c>
       <c r="Q220" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="R220" t="s">
         <v>25</v>
@@ -13790,13 +13787,13 @@
         <v>35</v>
       </c>
       <c r="D221" t="s">
+        <v>324</v>
+      </c>
+      <c r="E221" t="s">
+        <v>22</v>
+      </c>
+      <c r="F221" t="s">
         <v>325</v>
-      </c>
-      <c r="E221" t="s">
-        <v>40</v>
-      </c>
-      <c r="F221" t="s">
-        <v>326</v>
       </c>
       <c r="G221" t="s">
         <v>24</v>
@@ -13823,13 +13820,13 @@
         <v>25</v>
       </c>
       <c r="O221" t="s">
-        <v>27</v>
+        <v>42</v>
       </c>
       <c r="P221" t="s">
         <v>79</v>
       </c>
       <c r="Q221" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="R221" t="s">
         <v>25</v>
@@ -13846,13 +13843,13 @@
         <v>35</v>
       </c>
       <c r="D222" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="E222" t="s">
         <v>22</v>
       </c>
       <c r="F222" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="G222" t="s">
         <v>24</v>
@@ -13879,13 +13876,13 @@
         <v>25</v>
       </c>
       <c r="O222" t="s">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="P222" t="s">
         <v>79</v>
       </c>
       <c r="Q222" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="R222" t="s">
         <v>25</v>
@@ -13902,13 +13899,13 @@
         <v>35</v>
       </c>
       <c r="D223" t="s">
+        <v>324</v>
+      </c>
+      <c r="E223" t="s">
+        <v>35</v>
+      </c>
+      <c r="F223" t="s">
         <v>325</v>
-      </c>
-      <c r="E223" t="s">
-        <v>22</v>
-      </c>
-      <c r="F223" t="s">
-        <v>326</v>
       </c>
       <c r="G223" t="s">
         <v>24</v>
@@ -13926,22 +13923,22 @@
         <v>86</v>
       </c>
       <c r="L223" t="s">
-        <v>96</v>
+        <v>87</v>
       </c>
       <c r="M223" t="s">
-        <v>97</v>
+        <v>88</v>
       </c>
       <c r="N223" t="s">
         <v>25</v>
       </c>
       <c r="O223" t="s">
-        <v>51</v>
+        <v>27</v>
       </c>
       <c r="P223" t="s">
         <v>79</v>
       </c>
       <c r="Q223" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="R223" t="s">
         <v>25</v>
@@ -13958,13 +13955,13 @@
         <v>35</v>
       </c>
       <c r="D224" t="s">
+        <v>324</v>
+      </c>
+      <c r="E224" t="s">
+        <v>59</v>
+      </c>
+      <c r="F224" t="s">
         <v>325</v>
-      </c>
-      <c r="E224" t="s">
-        <v>35</v>
-      </c>
-      <c r="F224" t="s">
-        <v>326</v>
       </c>
       <c r="G224" t="s">
         <v>24</v>
@@ -13991,13 +13988,13 @@
         <v>25</v>
       </c>
       <c r="O224" t="s">
-        <v>27</v>
+        <v>42</v>
       </c>
       <c r="P224" t="s">
         <v>79</v>
       </c>
       <c r="Q224" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="R224" t="s">
         <v>25</v>
@@ -14014,13 +14011,13 @@
         <v>35</v>
       </c>
       <c r="D225" t="s">
+        <v>324</v>
+      </c>
+      <c r="E225" t="s">
+        <v>35</v>
+      </c>
+      <c r="F225" t="s">
         <v>325</v>
-      </c>
-      <c r="E225" t="s">
-        <v>59</v>
-      </c>
-      <c r="F225" t="s">
-        <v>326</v>
       </c>
       <c r="G225" t="s">
         <v>24</v>
@@ -14047,13 +14044,13 @@
         <v>25</v>
       </c>
       <c r="O225" t="s">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="P225" t="s">
         <v>79</v>
       </c>
       <c r="Q225" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="R225" t="s">
         <v>25</v>
@@ -14070,13 +14067,13 @@
         <v>35</v>
       </c>
       <c r="D226" t="s">
+        <v>324</v>
+      </c>
+      <c r="E226" t="s">
+        <v>35</v>
+      </c>
+      <c r="F226" t="s">
         <v>325</v>
-      </c>
-      <c r="E226" t="s">
-        <v>35</v>
-      </c>
-      <c r="F226" t="s">
-        <v>326</v>
       </c>
       <c r="G226" t="s">
         <v>24</v>
@@ -14088,28 +14085,28 @@
         <v>26</v>
       </c>
       <c r="J226" t="s">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="K226" t="s">
-        <v>86</v>
+        <v>104</v>
       </c>
       <c r="L226" t="s">
-        <v>87</v>
+        <v>105</v>
       </c>
       <c r="M226" t="s">
-        <v>88</v>
+        <v>106</v>
       </c>
       <c r="N226" t="s">
         <v>25</v>
       </c>
       <c r="O226" t="s">
-        <v>51</v>
+        <v>27</v>
       </c>
       <c r="P226" t="s">
         <v>79</v>
       </c>
       <c r="Q226" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="R226" t="s">
         <v>25</v>
@@ -14126,13 +14123,13 @@
         <v>35</v>
       </c>
       <c r="D227" t="s">
+        <v>324</v>
+      </c>
+      <c r="E227" t="s">
+        <v>35</v>
+      </c>
+      <c r="F227" t="s">
         <v>325</v>
-      </c>
-      <c r="E227" t="s">
-        <v>35</v>
-      </c>
-      <c r="F227" t="s">
-        <v>326</v>
       </c>
       <c r="G227" t="s">
         <v>24</v>
@@ -14159,13 +14156,13 @@
         <v>25</v>
       </c>
       <c r="O227" t="s">
-        <v>27</v>
+        <v>42</v>
       </c>
       <c r="P227" t="s">
         <v>79</v>
       </c>
       <c r="Q227" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="R227" t="s">
         <v>25</v>
@@ -14182,13 +14179,13 @@
         <v>35</v>
       </c>
       <c r="D228" t="s">
+        <v>324</v>
+      </c>
+      <c r="E228" t="s">
+        <v>40</v>
+      </c>
+      <c r="F228" t="s">
         <v>325</v>
-      </c>
-      <c r="E228" t="s">
-        <v>35</v>
-      </c>
-      <c r="F228" t="s">
-        <v>326</v>
       </c>
       <c r="G228" t="s">
         <v>24</v>
@@ -14215,13 +14212,13 @@
         <v>25</v>
       </c>
       <c r="O228" t="s">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="P228" t="s">
         <v>79</v>
       </c>
       <c r="Q228" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="R228" t="s">
         <v>25</v>
@@ -14238,13 +14235,13 @@
         <v>35</v>
       </c>
       <c r="D229" t="s">
+        <v>324</v>
+      </c>
+      <c r="E229" t="s">
+        <v>22</v>
+      </c>
+      <c r="F229" t="s">
         <v>325</v>
-      </c>
-      <c r="E229" t="s">
-        <v>40</v>
-      </c>
-      <c r="F229" t="s">
-        <v>326</v>
       </c>
       <c r="G229" t="s">
         <v>24</v>
@@ -14259,25 +14256,25 @@
         <v>51</v>
       </c>
       <c r="K229" t="s">
-        <v>104</v>
+        <v>56</v>
       </c>
       <c r="L229" t="s">
-        <v>105</v>
+        <v>114</v>
       </c>
       <c r="M229" t="s">
-        <v>106</v>
+        <v>118</v>
       </c>
       <c r="N229" t="s">
         <v>25</v>
       </c>
       <c r="O229" t="s">
-        <v>51</v>
+        <v>27</v>
       </c>
       <c r="P229" t="s">
         <v>79</v>
       </c>
       <c r="Q229" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="R229" t="s">
         <v>25</v>
@@ -14294,13 +14291,13 @@
         <v>35</v>
       </c>
       <c r="D230" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="E230" t="s">
         <v>22</v>
       </c>
       <c r="F230" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="G230" t="s">
         <v>24</v>
@@ -14327,13 +14324,13 @@
         <v>25</v>
       </c>
       <c r="O230" t="s">
-        <v>27</v>
+        <v>42</v>
       </c>
       <c r="P230" t="s">
         <v>79</v>
       </c>
       <c r="Q230" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="R230" t="s">
         <v>25</v>
@@ -14350,13 +14347,13 @@
         <v>35</v>
       </c>
       <c r="D231" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="E231" t="s">
         <v>22</v>
       </c>
       <c r="F231" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="G231" t="s">
         <v>24</v>
@@ -14383,13 +14380,13 @@
         <v>25</v>
       </c>
       <c r="O231" t="s">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="P231" t="s">
         <v>79</v>
       </c>
       <c r="Q231" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="R231" t="s">
         <v>25</v>
@@ -14406,46 +14403,46 @@
         <v>35</v>
       </c>
       <c r="D232" t="s">
+        <v>324</v>
+      </c>
+      <c r="E232" t="s">
+        <v>40</v>
+      </c>
+      <c r="F232" t="s">
         <v>325</v>
-      </c>
-      <c r="E232" t="s">
-        <v>22</v>
-      </c>
-      <c r="F232" t="s">
-        <v>326</v>
       </c>
       <c r="G232" t="s">
         <v>24</v>
       </c>
       <c r="H232" t="s">
-        <v>123</v>
+        <v>78</v>
       </c>
       <c r="I232" t="s">
         <v>26</v>
       </c>
       <c r="J232" t="s">
-        <v>51</v>
+        <v>27</v>
       </c>
       <c r="K232" t="s">
-        <v>56</v>
+        <v>28</v>
       </c>
       <c r="L232" t="s">
-        <v>114</v>
+        <v>82</v>
       </c>
       <c r="M232" t="s">
-        <v>118</v>
+        <v>83</v>
       </c>
       <c r="N232" t="s">
         <v>25</v>
       </c>
       <c r="O232" t="s">
-        <v>51</v>
+        <v>42</v>
       </c>
       <c r="P232" t="s">
         <v>79</v>
       </c>
       <c r="Q232" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="R232" t="s">
         <v>25</v>
@@ -14462,13 +14459,13 @@
         <v>35</v>
       </c>
       <c r="D233" t="s">
+        <v>324</v>
+      </c>
+      <c r="E233" t="s">
+        <v>22</v>
+      </c>
+      <c r="F233" t="s">
         <v>325</v>
-      </c>
-      <c r="E233" t="s">
-        <v>40</v>
-      </c>
-      <c r="F233" t="s">
-        <v>326</v>
       </c>
       <c r="G233" t="s">
         <v>24</v>
@@ -14495,13 +14492,13 @@
         <v>25</v>
       </c>
       <c r="O233" t="s">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="P233" t="s">
         <v>79</v>
       </c>
       <c r="Q233" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="R233" t="s">
         <v>25</v>
@@ -14518,13 +14515,13 @@
         <v>35</v>
       </c>
       <c r="D234" t="s">
+        <v>324</v>
+      </c>
+      <c r="E234" t="s">
+        <v>40</v>
+      </c>
+      <c r="F234" t="s">
         <v>325</v>
-      </c>
-      <c r="E234" t="s">
-        <v>22</v>
-      </c>
-      <c r="F234" t="s">
-        <v>326</v>
       </c>
       <c r="G234" t="s">
         <v>24</v>
@@ -14536,28 +14533,28 @@
         <v>26</v>
       </c>
       <c r="J234" t="s">
+        <v>42</v>
+      </c>
+      <c r="K234" t="s">
+        <v>86</v>
+      </c>
+      <c r="L234" t="s">
+        <v>96</v>
+      </c>
+      <c r="M234" t="s">
+        <v>97</v>
+      </c>
+      <c r="N234" t="s">
+        <v>25</v>
+      </c>
+      <c r="O234" t="s">
         <v>27</v>
       </c>
-      <c r="K234" t="s">
-        <v>28</v>
-      </c>
-      <c r="L234" t="s">
-        <v>82</v>
-      </c>
-      <c r="M234" t="s">
-        <v>83</v>
-      </c>
-      <c r="N234" t="s">
-        <v>25</v>
-      </c>
-      <c r="O234" t="s">
-        <v>51</v>
-      </c>
       <c r="P234" t="s">
         <v>79</v>
       </c>
       <c r="Q234" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="R234" t="s">
         <v>25</v>
@@ -14574,13 +14571,13 @@
         <v>35</v>
       </c>
       <c r="D235" t="s">
+        <v>324</v>
+      </c>
+      <c r="E235" t="s">
+        <v>22</v>
+      </c>
+      <c r="F235" t="s">
         <v>325</v>
-      </c>
-      <c r="E235" t="s">
-        <v>40</v>
-      </c>
-      <c r="F235" t="s">
-        <v>326</v>
       </c>
       <c r="G235" t="s">
         <v>24</v>
@@ -14607,13 +14604,13 @@
         <v>25</v>
       </c>
       <c r="O235" t="s">
-        <v>27</v>
+        <v>42</v>
       </c>
       <c r="P235" t="s">
         <v>79</v>
       </c>
       <c r="Q235" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="R235" t="s">
         <v>25</v>
@@ -14630,13 +14627,13 @@
         <v>35</v>
       </c>
       <c r="D236" t="s">
+        <v>324</v>
+      </c>
+      <c r="E236" t="s">
+        <v>40</v>
+      </c>
+      <c r="F236" t="s">
         <v>325</v>
-      </c>
-      <c r="E236" t="s">
-        <v>22</v>
-      </c>
-      <c r="F236" t="s">
-        <v>326</v>
       </c>
       <c r="G236" t="s">
         <v>24</v>
@@ -14663,13 +14660,13 @@
         <v>25</v>
       </c>
       <c r="O236" t="s">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="P236" t="s">
         <v>79</v>
       </c>
       <c r="Q236" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="R236" t="s">
         <v>25</v>
@@ -14686,13 +14683,13 @@
         <v>35</v>
       </c>
       <c r="D237" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="E237" t="s">
         <v>40</v>
       </c>
       <c r="F237" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="G237" t="s">
         <v>24</v>
@@ -14710,22 +14707,22 @@
         <v>86</v>
       </c>
       <c r="L237" t="s">
-        <v>96</v>
+        <v>87</v>
       </c>
       <c r="M237" t="s">
-        <v>97</v>
+        <v>88</v>
       </c>
       <c r="N237" t="s">
         <v>25</v>
       </c>
       <c r="O237" t="s">
-        <v>51</v>
+        <v>27</v>
       </c>
       <c r="P237" t="s">
         <v>79</v>
       </c>
       <c r="Q237" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="R237" t="s">
         <v>25</v>
@@ -14742,13 +14739,13 @@
         <v>35</v>
       </c>
       <c r="D238" t="s">
+        <v>324</v>
+      </c>
+      <c r="E238" t="s">
+        <v>35</v>
+      </c>
+      <c r="F238" t="s">
         <v>325</v>
-      </c>
-      <c r="E238" t="s">
-        <v>40</v>
-      </c>
-      <c r="F238" t="s">
-        <v>326</v>
       </c>
       <c r="G238" t="s">
         <v>24</v>
@@ -14775,13 +14772,13 @@
         <v>25</v>
       </c>
       <c r="O238" t="s">
-        <v>27</v>
+        <v>42</v>
       </c>
       <c r="P238" t="s">
         <v>79</v>
       </c>
       <c r="Q238" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="R238" t="s">
         <v>25</v>
@@ -14798,13 +14795,13 @@
         <v>35</v>
       </c>
       <c r="D239" t="s">
+        <v>324</v>
+      </c>
+      <c r="E239" t="s">
+        <v>40</v>
+      </c>
+      <c r="F239" t="s">
         <v>325</v>
-      </c>
-      <c r="E239" t="s">
-        <v>35</v>
-      </c>
-      <c r="F239" t="s">
-        <v>326</v>
       </c>
       <c r="G239" t="s">
         <v>24</v>
@@ -14831,13 +14828,13 @@
         <v>25</v>
       </c>
       <c r="O239" t="s">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="P239" t="s">
         <v>79</v>
       </c>
       <c r="Q239" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="R239" t="s">
         <v>25</v>
@@ -14854,13 +14851,13 @@
         <v>35</v>
       </c>
       <c r="D240" t="s">
+        <v>324</v>
+      </c>
+      <c r="E240" t="s">
+        <v>22</v>
+      </c>
+      <c r="F240" t="s">
         <v>325</v>
-      </c>
-      <c r="E240" t="s">
-        <v>40</v>
-      </c>
-      <c r="F240" t="s">
-        <v>326</v>
       </c>
       <c r="G240" t="s">
         <v>24</v>
@@ -14872,28 +14869,28 @@
         <v>26</v>
       </c>
       <c r="J240" t="s">
+        <v>51</v>
+      </c>
+      <c r="K240" t="s">
+        <v>104</v>
+      </c>
+      <c r="L240" t="s">
+        <v>105</v>
+      </c>
+      <c r="M240" t="s">
+        <v>106</v>
+      </c>
+      <c r="N240" t="s">
+        <v>25</v>
+      </c>
+      <c r="O240" t="s">
         <v>42</v>
       </c>
-      <c r="K240" t="s">
-        <v>86</v>
-      </c>
-      <c r="L240" t="s">
-        <v>87</v>
-      </c>
-      <c r="M240" t="s">
-        <v>88</v>
-      </c>
-      <c r="N240" t="s">
-        <v>25</v>
-      </c>
-      <c r="O240" t="s">
-        <v>51</v>
-      </c>
       <c r="P240" t="s">
         <v>79</v>
       </c>
       <c r="Q240" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="R240" t="s">
         <v>25</v>
@@ -14910,13 +14907,13 @@
         <v>35</v>
       </c>
       <c r="D241" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="E241" t="s">
         <v>22</v>
       </c>
       <c r="F241" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="G241" t="s">
         <v>24</v>
@@ -14943,13 +14940,13 @@
         <v>25</v>
       </c>
       <c r="O241" t="s">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="P241" t="s">
         <v>79</v>
       </c>
       <c r="Q241" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="R241" t="s">
         <v>25</v>
@@ -14966,13 +14963,13 @@
         <v>35</v>
       </c>
       <c r="D242" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="E242" t="s">
         <v>22</v>
       </c>
       <c r="F242" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="G242" t="s">
         <v>24</v>
@@ -14987,25 +14984,25 @@
         <v>51</v>
       </c>
       <c r="K242" t="s">
-        <v>104</v>
+        <v>56</v>
       </c>
       <c r="L242" t="s">
-        <v>105</v>
+        <v>114</v>
       </c>
       <c r="M242" t="s">
-        <v>106</v>
+        <v>118</v>
       </c>
       <c r="N242" t="s">
         <v>25</v>
       </c>
       <c r="O242" t="s">
-        <v>51</v>
+        <v>27</v>
       </c>
       <c r="P242" t="s">
         <v>79</v>
       </c>
       <c r="Q242" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="R242" t="s">
         <v>25</v>
@@ -15022,13 +15019,13 @@
         <v>35</v>
       </c>
       <c r="D243" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="E243" t="s">
         <v>22</v>
       </c>
       <c r="F243" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="G243" t="s">
         <v>24</v>
@@ -15055,13 +15052,13 @@
         <v>25</v>
       </c>
       <c r="O243" t="s">
-        <v>27</v>
+        <v>42</v>
       </c>
       <c r="P243" t="s">
         <v>79</v>
       </c>
       <c r="Q243" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="R243" t="s">
         <v>25</v>
@@ -15078,13 +15075,13 @@
         <v>35</v>
       </c>
       <c r="D244" t="s">
+        <v>324</v>
+      </c>
+      <c r="E244" t="s">
+        <v>40</v>
+      </c>
+      <c r="F244" t="s">
         <v>325</v>
-      </c>
-      <c r="E244" t="s">
-        <v>22</v>
-      </c>
-      <c r="F244" t="s">
-        <v>326</v>
       </c>
       <c r="G244" t="s">
         <v>24</v>
@@ -15111,13 +15108,13 @@
         <v>25</v>
       </c>
       <c r="O244" t="s">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="P244" t="s">
         <v>79</v>
       </c>
       <c r="Q244" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="R244" t="s">
         <v>25</v>
@@ -15131,57 +15128,57 @@
         <v>19</v>
       </c>
       <c r="C245" t="s">
-        <v>35</v>
+        <v>19</v>
       </c>
       <c r="D245" t="s">
-        <v>325</v>
+        <v>75</v>
       </c>
       <c r="E245" t="s">
-        <v>40</v>
+        <v>22</v>
       </c>
       <c r="F245" t="s">
-        <v>326</v>
+        <v>354</v>
       </c>
       <c r="G245" t="s">
-        <v>24</v>
+        <v>355</v>
       </c>
       <c r="H245" t="s">
         <v>78</v>
       </c>
       <c r="I245" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="J245" t="s">
-        <v>51</v>
+        <v>25</v>
       </c>
       <c r="K245" t="s">
-        <v>56</v>
+        <v>25</v>
       </c>
       <c r="L245" t="s">
-        <v>114</v>
+        <v>25</v>
       </c>
       <c r="M245" t="s">
-        <v>118</v>
+        <v>25</v>
       </c>
       <c r="N245" t="s">
         <v>25</v>
       </c>
       <c r="O245" t="s">
-        <v>51</v>
+        <v>25</v>
       </c>
       <c r="P245" t="s">
         <v>79</v>
       </c>
       <c r="Q245" t="s">
-        <v>326</v>
+        <v>25</v>
       </c>
       <c r="R245" t="s">
-        <v>25</v>
+        <v>76</v>
       </c>
     </row>
     <row r="246">
       <c r="A246" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="B246" t="s">
         <v>19</v>
@@ -15190,34 +15187,34 @@
         <v>19</v>
       </c>
       <c r="D246" t="s">
-        <v>75</v>
+        <v>121</v>
       </c>
       <c r="E246" t="s">
-        <v>22</v>
+        <v>59</v>
       </c>
       <c r="F246" t="s">
-        <v>355</v>
+        <v>122</v>
       </c>
       <c r="G246" t="s">
-        <v>356</v>
+        <v>77</v>
       </c>
       <c r="H246" t="s">
-        <v>78</v>
+        <v>123</v>
       </c>
       <c r="I246" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="J246" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="K246" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="L246" t="s">
-        <v>25</v>
+        <v>82</v>
       </c>
       <c r="M246" t="s">
-        <v>25</v>
+        <v>83</v>
       </c>
       <c r="N246" t="s">
         <v>25</v>
@@ -15229,10 +15226,10 @@
         <v>79</v>
       </c>
       <c r="Q246" t="s">
-        <v>25</v>
+        <v>122</v>
       </c>
       <c r="R246" t="s">
-        <v>76</v>
+        <v>122</v>
       </c>
     </row>
     <row r="247">
@@ -15264,16 +15261,16 @@
         <v>26</v>
       </c>
       <c r="J247" t="s">
-        <v>27</v>
+        <v>42</v>
       </c>
       <c r="K247" t="s">
-        <v>28</v>
+        <v>86</v>
       </c>
       <c r="L247" t="s">
-        <v>82</v>
+        <v>96</v>
       </c>
       <c r="M247" t="s">
-        <v>83</v>
+        <v>97</v>
       </c>
       <c r="N247" t="s">
         <v>25</v>
@@ -15305,7 +15302,7 @@
         <v>121</v>
       </c>
       <c r="E248" t="s">
-        <v>59</v>
+        <v>22</v>
       </c>
       <c r="F248" t="s">
         <v>122</v>
@@ -15320,16 +15317,16 @@
         <v>26</v>
       </c>
       <c r="J248" t="s">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="K248" t="s">
-        <v>86</v>
+        <v>104</v>
       </c>
       <c r="L248" t="s">
-        <v>96</v>
+        <v>105</v>
       </c>
       <c r="M248" t="s">
-        <v>97</v>
+        <v>106</v>
       </c>
       <c r="N248" t="s">
         <v>25</v>
@@ -15361,7 +15358,7 @@
         <v>121</v>
       </c>
       <c r="E249" t="s">
-        <v>22</v>
+        <v>59</v>
       </c>
       <c r="F249" t="s">
         <v>122</v>
@@ -15379,13 +15376,13 @@
         <v>51</v>
       </c>
       <c r="K249" t="s">
-        <v>104</v>
+        <v>56</v>
       </c>
       <c r="L249" t="s">
-        <v>105</v>
+        <v>114</v>
       </c>
       <c r="M249" t="s">
-        <v>106</v>
+        <v>118</v>
       </c>
       <c r="N249" t="s">
         <v>25</v>
@@ -15417,7 +15414,7 @@
         <v>121</v>
       </c>
       <c r="E250" t="s">
-        <v>59</v>
+        <v>35</v>
       </c>
       <c r="F250" t="s">
         <v>122</v>
@@ -15426,22 +15423,22 @@
         <v>77</v>
       </c>
       <c r="H250" t="s">
-        <v>123</v>
+        <v>78</v>
       </c>
       <c r="I250" t="s">
         <v>26</v>
       </c>
       <c r="J250" t="s">
-        <v>51</v>
+        <v>27</v>
       </c>
       <c r="K250" t="s">
-        <v>56</v>
+        <v>28</v>
       </c>
       <c r="L250" t="s">
-        <v>114</v>
+        <v>82</v>
       </c>
       <c r="M250" t="s">
-        <v>118</v>
+        <v>83</v>
       </c>
       <c r="N250" t="s">
         <v>25</v>
@@ -15488,16 +15485,16 @@
         <v>26</v>
       </c>
       <c r="J251" t="s">
-        <v>27</v>
+        <v>51</v>
       </c>
       <c r="K251" t="s">
-        <v>28</v>
+        <v>104</v>
       </c>
       <c r="L251" t="s">
-        <v>82</v>
+        <v>105</v>
       </c>
       <c r="M251" t="s">
-        <v>83</v>
+        <v>106</v>
       </c>
       <c r="N251" t="s">
         <v>25</v>
@@ -15529,7 +15526,7 @@
         <v>121</v>
       </c>
       <c r="E252" t="s">
-        <v>35</v>
+        <v>59</v>
       </c>
       <c r="F252" t="s">
         <v>122</v>
@@ -15544,16 +15541,16 @@
         <v>26</v>
       </c>
       <c r="J252" t="s">
-        <v>51</v>
+        <v>42</v>
       </c>
       <c r="K252" t="s">
-        <v>104</v>
+        <v>86</v>
       </c>
       <c r="L252" t="s">
-        <v>105</v>
+        <v>87</v>
       </c>
       <c r="M252" t="s">
-        <v>106</v>
+        <v>88</v>
       </c>
       <c r="N252" t="s">
         <v>25</v>
@@ -15585,7 +15582,7 @@
         <v>121</v>
       </c>
       <c r="E253" t="s">
-        <v>59</v>
+        <v>22</v>
       </c>
       <c r="F253" t="s">
         <v>122</v>
@@ -15600,16 +15597,16 @@
         <v>26</v>
       </c>
       <c r="J253" t="s">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="K253" t="s">
-        <v>86</v>
+        <v>56</v>
       </c>
       <c r="L253" t="s">
-        <v>87</v>
+        <v>114</v>
       </c>
       <c r="M253" t="s">
-        <v>88</v>
+        <v>118</v>
       </c>
       <c r="N253" t="s">
         <v>25</v>
@@ -15638,7 +15635,7 @@
         <v>19</v>
       </c>
       <c r="D254" t="s">
-        <v>121</v>
+        <v>139</v>
       </c>
       <c r="E254" t="s">
         <v>22</v>
@@ -15650,22 +15647,22 @@
         <v>77</v>
       </c>
       <c r="H254" t="s">
-        <v>78</v>
+        <v>123</v>
       </c>
       <c r="I254" t="s">
-        <v>26</v>
+        <v>140</v>
       </c>
       <c r="J254" t="s">
-        <v>51</v>
+        <v>42</v>
       </c>
       <c r="K254" t="s">
-        <v>56</v>
+        <v>25</v>
       </c>
       <c r="L254" t="s">
-        <v>114</v>
+        <v>25</v>
       </c>
       <c r="M254" t="s">
-        <v>118</v>
+        <v>25</v>
       </c>
       <c r="N254" t="s">
         <v>25</v>
@@ -15674,7 +15671,7 @@
         <v>25</v>
       </c>
       <c r="P254" t="s">
-        <v>79</v>
+        <v>141</v>
       </c>
       <c r="Q254" t="s">
         <v>122</v>
@@ -15706,13 +15703,13 @@
         <v>77</v>
       </c>
       <c r="H255" t="s">
-        <v>123</v>
+        <v>78</v>
       </c>
       <c r="I255" t="s">
         <v>140</v>
       </c>
       <c r="J255" t="s">
-        <v>42</v>
+        <v>27</v>
       </c>
       <c r="K255" t="s">
         <v>25</v>
@@ -15753,7 +15750,7 @@
         <v>139</v>
       </c>
       <c r="E256" t="s">
-        <v>22</v>
+        <v>40</v>
       </c>
       <c r="F256" t="s">
         <v>122</v>
@@ -15768,7 +15765,7 @@
         <v>140</v>
       </c>
       <c r="J256" t="s">
-        <v>27</v>
+        <v>42</v>
       </c>
       <c r="K256" t="s">
         <v>25</v>
@@ -15803,37 +15800,37 @@
         <v>19</v>
       </c>
       <c r="C257" t="s">
-        <v>19</v>
+        <v>59</v>
       </c>
       <c r="D257" t="s">
-        <v>139</v>
+        <v>368</v>
       </c>
       <c r="E257" t="s">
-        <v>40</v>
+        <v>19</v>
       </c>
       <c r="F257" t="s">
-        <v>122</v>
+        <v>239</v>
       </c>
       <c r="G257" t="s">
         <v>77</v>
       </c>
       <c r="H257" t="s">
-        <v>78</v>
+        <v>25</v>
       </c>
       <c r="I257" t="s">
-        <v>140</v>
+        <v>26</v>
       </c>
       <c r="J257" t="s">
         <v>42</v>
       </c>
       <c r="K257" t="s">
-        <v>25</v>
+        <v>86</v>
       </c>
       <c r="L257" t="s">
-        <v>25</v>
+        <v>87</v>
       </c>
       <c r="M257" t="s">
-        <v>25</v>
+        <v>88</v>
       </c>
       <c r="N257" t="s">
         <v>25</v>
@@ -15842,18 +15839,18 @@
         <v>25</v>
       </c>
       <c r="P257" t="s">
-        <v>141</v>
+        <v>369</v>
       </c>
       <c r="Q257" t="s">
-        <v>122</v>
+        <v>240</v>
       </c>
       <c r="R257" t="s">
-        <v>122</v>
+        <v>25</v>
       </c>
     </row>
     <row r="258">
       <c r="A258" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="B258" t="s">
         <v>19</v>
@@ -15862,7 +15859,7 @@
         <v>59</v>
       </c>
       <c r="D258" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="E258" t="s">
         <v>19</v>
@@ -15898,7 +15895,7 @@
         <v>25</v>
       </c>
       <c r="P258" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="Q258" t="s">
         <v>240</v>
@@ -15918,13 +15915,13 @@
         <v>59</v>
       </c>
       <c r="D259" t="s">
-        <v>369</v>
+        <v>302</v>
       </c>
       <c r="E259" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="F259" t="s">
-        <v>239</v>
+        <v>182</v>
       </c>
       <c r="G259" t="s">
         <v>77</v>
@@ -15936,16 +15933,16 @@
         <v>26</v>
       </c>
       <c r="J259" t="s">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="K259" t="s">
-        <v>86</v>
+        <v>104</v>
       </c>
       <c r="L259" t="s">
-        <v>87</v>
+        <v>105</v>
       </c>
       <c r="M259" t="s">
-        <v>88</v>
+        <v>106</v>
       </c>
       <c r="N259" t="s">
         <v>25</v>
@@ -15954,68 +15951,12 @@
         <v>25</v>
       </c>
       <c r="P259" t="s">
-        <v>370</v>
+        <v>303</v>
       </c>
       <c r="Q259" t="s">
-        <v>240</v>
+        <v>183</v>
       </c>
       <c r="R259" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="260">
-      <c r="A260" t="s">
-        <v>372</v>
-      </c>
-      <c r="B260" t="s">
-        <v>19</v>
-      </c>
-      <c r="C260" t="s">
-        <v>59</v>
-      </c>
-      <c r="D260" t="s">
-        <v>303</v>
-      </c>
-      <c r="E260" t="s">
-        <v>22</v>
-      </c>
-      <c r="F260" t="s">
-        <v>182</v>
-      </c>
-      <c r="G260" t="s">
-        <v>77</v>
-      </c>
-      <c r="H260" t="s">
-        <v>25</v>
-      </c>
-      <c r="I260" t="s">
-        <v>26</v>
-      </c>
-      <c r="J260" t="s">
-        <v>51</v>
-      </c>
-      <c r="K260" t="s">
-        <v>104</v>
-      </c>
-      <c r="L260" t="s">
-        <v>105</v>
-      </c>
-      <c r="M260" t="s">
-        <v>106</v>
-      </c>
-      <c r="N260" t="s">
-        <v>25</v>
-      </c>
-      <c r="O260" t="s">
-        <v>25</v>
-      </c>
-      <c r="P260" t="s">
-        <v>304</v>
-      </c>
-      <c r="Q260" t="s">
-        <v>183</v>
-      </c>
-      <c r="R260" t="s">
         <v>183</v>
       </c>
     </row>

</xml_diff>